<commit_message>
updated failed test cases
</commit_message>
<xml_diff>
--- a/src/main/resources/PotentialReviewersContact_Field_Values.xlsx
+++ b/src/main/resources/PotentialReviewersContact_Field_Values.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="21601"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="21901"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Dev\govgrants-product-automation\src\main\resources\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F8591E05-22CE-40EF-9503-DC4B7F2D39D1}" xr6:coauthVersionLast="43" xr6:coauthVersionMax="43" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{59C1491E-9A2F-478C-B0D3-8FE7DB561749}" xr6:coauthVersionLast="43" xr6:coauthVersionMax="43" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="1500" yWindow="1500" windowWidth="17280" windowHeight="8964" activeTab="1" xr2:uid="{FE4041C9-411E-47B8-A648-17C164901997}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12576" xr2:uid="{FE4041C9-411E-47B8-A648-17C164901997}"/>
   </bookViews>
   <sheets>
     <sheet name="Creation" sheetId="1" r:id="rId1"/>

</xml_diff>

<commit_message>
Merged PR 2957: Merge Deepika_prod to master
Automated 3 new test cases - @57840, @57839, @57838                                                                                                                                        Fixed failed Test Cases in SIte Visits and Desk Review
Added Deletion API for DUNS and Contact related Test Cases
</commit_message>
<xml_diff>
--- a/src/main/resources/PotentialReviewersContact_Field_Values.xlsx
+++ b/src/main/resources/PotentialReviewersContact_Field_Values.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="21601"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="21901"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Dev\govgrants-product-automation\src\main\resources\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F8591E05-22CE-40EF-9503-DC4B7F2D39D1}" xr6:coauthVersionLast="43" xr6:coauthVersionMax="43" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{59C1491E-9A2F-478C-B0D3-8FE7DB561749}" xr6:coauthVersionLast="43" xr6:coauthVersionMax="43" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="1500" yWindow="1500" windowWidth="17280" windowHeight="8964" activeTab="1" xr2:uid="{FE4041C9-411E-47B8-A648-17C164901997}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12576" xr2:uid="{FE4041C9-411E-47B8-A648-17C164901997}"/>
   </bookViews>
   <sheets>
     <sheet name="Creation" sheetId="1" r:id="rId1"/>

</xml_diff>